<commit_message>
Fix Workday workbook validation and readiness evidence
Handle corrupt workbook members as validation errors, expose supported administrator answers, and keep uncollected network attestations out of guided readiness profiles. Add regressions and regenerate the Workday workbook.

Copilot-Session: aecd8af3-0d46-4d05-a26d-6b4dd3f05688
</commit_message>
<xml_diff>
--- a/solutions/ess-maker-skills/src/skills/setup/workday-da/assets/workday-admin-handoff.xlsx
+++ b/solutions/ess-maker-skills/src/skills/setup/workday-da/assets/workday-admin-handoff.xlsx
@@ -525,7 +525,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirm the policy applies to the ESS OAuth client identity and allows SAML for the intended employees. Record whether that rule was already active or a reviewed policy was activated.</t>
+          <t xml:space="preserve">Confirm the policy applies to the ESS OAuth client identity and allows SAML for the intended employees. Enter exactly one of: An existing active policy scopes the ESS OAuth client and allows SAML for the intended employees; A reviewed policy scoped to the ESS OAuth client was activated</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record the configured employee population.</t>
+          <t xml:space="preserve">Record the configured employee population. Enter exactly one of: Entire workforce - All Employees access is configured; Limited or test population - the intended Workday security group and test employee access are configured</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">

</xml_diff>